<commit_message>
feat: record test execution results, add EC-04, and update execution plan for HW01 Req 3
- Record FAIL results for TC-W03 (asymmetric sweep), TC-W05 (jerking oscillation), EC-04 (mid-sweep direction reversal from rapid SPEED pulls)
- Add EC-04 edge case to test_cases.md, test_cases.xlsx, and test_case_checklist.xlsx
- Renumber TC IDs to fill gaps: TC-S05→TC-S04, TC-S06→TC-S05, TC-W07→TC-W05
- Update video execution plan: TC-S03, TC-W01, TC-T01 (PASS) + TC-W03, TC-W05 (FAIL)
</commit_message>
<xml_diff>
--- a/homeworks/HW01/artifacts/physical-product-testing/test_cases.xlsx
+++ b/homeworks/HW01/artifacts/physical-product-testing/test_cases.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="115">
   <si>
     <t xml:space="preserve">Test Cases — Senko TC1626 Wall-mounted Fan</t>
   </si>
@@ -65,6 +65,12 @@
     <t xml:space="preserve">Motor runs at Level 1 (lowest speed).</t>
   </si>
   <si>
+    <t xml:space="preserve">Motor runs at Level 1 with highest speed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FAIL</t>
+  </si>
+  <si>
     <t xml:space="preserve">TC-S02</t>
   </si>
   <si>
@@ -72,6 +78,117 @@
   </si>
   <si>
     <t xml:space="preserve">3 consecutive pulls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Fan at Level 0.
+2. Pull cord 3 times (one at a time).
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each pull advances one level; speed increases visibly at each step (Level 1 → 2 → 3).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each pull advances one level; but speed decreases visibly at each step (Level 1 → 2 → 3).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-S03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify loop-back to Level 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4th pull from Level 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Fan at Level 3.
+2. Pull SPEED cord once.
+Record video (≤ 60 s, voice narration required) as proof of execution.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fan returns to Level 0 (motor off).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fan returns to Level 0 (motor off)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PASS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-S04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify rapid successive pulls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 pulls within &lt; 1 second</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Fan at Level 0.
+2. Pull cord twice in rapid succession.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ratchet counts exactly 2 steps; stops at Level 2. No skipped or double-counted notch.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-S05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify partial-pull (incomplete stroke)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cord pulled to ~50% of travel, then released</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Fan at Level 0.
+2. Pull cord halfway, then release without completing the stroke.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ratchet does NOT advance to next level OR snaps back to rest position. No jammed-between-notch state.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A2 — Sub-system: SWING (left pull-cord, toggle oscillation on/off)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-W01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify oscillation starts on first pull</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 pull while swing is OFF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Fan running at Level 2; swing OFF.
+2. Pull SWING cord once.
+Record video (≤ 60 s, voice narration required) as proof of execution.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fan head begins left–right oscillation automatically.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-W02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify oscillation stops on second pull</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 pull while swing is ON</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Fan is oscillating.
+2. Pull SWING cord once.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fan head stops oscillating and holds its current angle.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-W03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify oscillation sweep range and symmetry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Observe 1 complete sweep cycle after enabling</t>
   </si>
   <si>
     <r>
@@ -81,8 +198,8 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">1. Fan at Level 0.
-2. Pull cord 3 times (one at a time).
+      <t xml:space="preserve">1. Enable swing.
+2. Observe one full left–right cycle.
 </t>
     </r>
     <r>
@@ -95,110 +212,12 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Each pull advances one level; speed increases visibly at each step (Level 1 → 2 → 3).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-S03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verify loop-back to Level 0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4th pull from Level 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Fan at Level 3.
-2. Pull SPEED cord once.
-Record video (≤ 60 s, voice narration required) as proof of execution.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fan returns to Level 0 (motor off).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-S05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verify rapid successive pulls</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2 pulls within &lt; 1 second</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Fan at Level 0.
-2. Pull cord twice in rapid succession.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ratchet counts exactly 2 steps; stops at Level 2. No skipped or double-counted notch.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-S06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verify partial-pull (incomplete stroke)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cord pulled to ~50% of travel, then released</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Fan at Level 0.
-2. Pull cord halfway, then release without completing the stroke.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ratchet does NOT advance to next level OR snaps back to rest position. No jammed-between-notch state.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A2 — Sub-system: SWING (left pull-cord, toggle oscillation on/off)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-W01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verify oscillation starts on first pull</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 pull while swing is OFF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Fan running at Level 2; swing OFF.
-2. Pull SWING cord once.
-Record video (≤ 60 s, voice narration required) as proof of execution.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fan head begins left–right oscillation automatically.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-W02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verify oscillation stops on second pull</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 pull while swing is ON</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Fan is oscillating.
-2. Pull SWING cord once.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fan head stops oscillating and holds its current angle.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-W03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verify oscillation sweep range and symmetry</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Observe 1 complete sweep cycle after enabling</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Enable swing.
-2. Observe one full left–right cycle.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Sweep is symmetrical on both sides; head reaches the designed angular limit on each side without stalling or overshooting.</t>
   </si>
   <si>
+    <t xml:space="preserve">Sweep is asymmetrical: amplitude deviates noticeably to the right (observer's perspective); right arc is wider than left arc.</t>
+  </si>
+  <si>
     <t xml:space="preserve">TC-W04</t>
   </si>
   <si>
@@ -208,14 +227,23 @@
     <t xml:space="preserve">Change SPEED level while swing is active</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Enable swing at Level 1.
-2. Pull SPEED cord to switch to Level 3.</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1. Enable swing at Level 1.
+2. Pull SPEED cord to switch to Level 3.
+</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">Oscillation continues uninterrupted; only airflow speed changes.</t>
   </si>
   <si>
-    <t xml:space="preserve">TC-W07</t>
+    <t xml:space="preserve">TC-W05</t>
   </si>
   <si>
     <t xml:space="preserve">Verify smooth and quiet oscillation</t>
@@ -224,11 +252,31 @@
     <t xml:space="preserve">Observe 10 oscillation cycles</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Enable swing.
-2. Listen and observe 10 complete cycles.</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1. Enable swing.
+2. Listen and observe 10 complete cycles.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">Record video (≤ 60 s, voice narration required) as proof of execution.</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">Motion is smooth with no jerking at reversal points; no abnormal noise (grinding, clicking) at direction changes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oscillation is not smooth: intermittent jerking observed during swap cycles.</t>
   </si>
   <si>
     <t xml:space="preserve">A3 — Sub-system: TILT (neck pivot detent, vertical angle adjustment)</t>
@@ -328,8 +376,7 @@
     <t xml:space="preserve">1. Set fan to Level 2.
 2. Disconnect power (unplug or cut circuit breaker).
 3. Wait 5 s.
-4. Restore power.
-Record video (≤ 60 s, voice narration required) as proof of execution.</t>
+4. Restore power.</t>
   </si>
   <si>
     <t xml:space="preserve">Fan restarts at Level 2 immediately (mechanical switch retains position). Behavior is documented and user is aware — no unexpected startup.</t>
@@ -367,6 +414,27 @@
   </si>
   <si>
     <t xml:space="preserve">All mounting screws and bracket remain tight; no audible rattle from the mount; no visible displacement of the fan from its original mounted position.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EC-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify oscillation direction is not reversed mid-sweep by rapid SPEED level transitions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SWING ON; SPEED cord pulled ≥ 3 times in rapid succession (~1 pull/second) while head is mid-sweep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Fan at Level 1, swing ON.
+2. Observe head is mid-sweep (not at a reversal point).
+3. Pull SPEED cord 3–4 times rapidly, completing at least one full cycle (1→2→3→0).
+4. Observe oscillation direction during and immediately after the speed transitions.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oscillation continues in its current direction until the natural mechanical reversal point; no mid-sweep direction reversal is triggered by SPEED level changes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fan head reversed oscillation direction mid-sweep during rapid SPEED level transitions before reaching the natural reversal point.</t>
   </si>
 </sst>
 </file>
@@ -376,7 +444,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -440,6 +508,12 @@
       <sz val="10"/>
       <name val="Calibri"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="7">
@@ -529,7 +603,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -563,6 +637,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -826,7 +904,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10"/>
@@ -834,11 +912,11 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="40"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="47.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="10"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -849,7 +927,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -872,7 +950,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
         <v>8</v>
       </c>
@@ -883,7 +961,7 @@
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
     </row>
-    <row r="4" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="20.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
         <v>9</v>
       </c>
@@ -899,88 +977,108 @@
       <c r="E4" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-    </row>
-    <row r="5" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F4" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="30.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B5" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="G5" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="F5" s="8"/>
-      <c r="G5" s="8"/>
-    </row>
-    <row r="6" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="6" customFormat="false" ht="40.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
-    </row>
-    <row r="7" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>26</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="20.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="E7" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G7" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-    </row>
-    <row r="8" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="8" customFormat="false" ht="30.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
-    </row>
-    <row r="9" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>38</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -989,104 +1087,124 @@
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
     </row>
-    <row r="10" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="40.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-    </row>
-    <row r="11" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>44</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="20.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
-    </row>
-    <row r="12" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>49</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="40.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-    </row>
-    <row r="13" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>54</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="30.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
-    </row>
-    <row r="14" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>60</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="40.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
-    </row>
-    <row r="15" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>65</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
@@ -1095,104 +1213,124 @@
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
     </row>
-    <row r="16" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="40.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
-    </row>
-    <row r="17" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>72</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="20.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="F17" s="8"/>
-      <c r="G17" s="8"/>
-    </row>
-    <row r="18" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>77</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="20.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
-    </row>
-    <row r="19" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>82</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="20.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
-    </row>
-    <row r="20" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>87</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="20.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="F20" s="6"/>
-      <c r="G20" s="6"/>
-    </row>
-    <row r="21" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>92</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
@@ -1201,62 +1339,97 @@
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
     </row>
-    <row r="22" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="B22" s="10" t="s">
-        <v>88</v>
-      </c>
-      <c r="C22" s="10" t="s">
-        <v>89</v>
-      </c>
-      <c r="D22" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="E22" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="F22" s="10"/>
-      <c r="G22" s="10"/>
-    </row>
-    <row r="23" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="B23" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="C23" s="10" t="s">
+    <row r="22" customFormat="false" ht="40.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="D23" s="10" t="s">
+      <c r="B22" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="E23" s="10" t="s">
+      <c r="C22" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="F23" s="10"/>
-      <c r="G23" s="10"/>
-    </row>
-    <row r="24" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="9" t="s">
+      <c r="D22" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="B24" s="10" t="s">
+      <c r="E22" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="C24" s="10" t="s">
+      <c r="F22" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="G22" s="11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="30.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="D24" s="10" t="s">
+      <c r="B23" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="E24" s="10" t="s">
+      <c r="C23" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="F24" s="10"/>
-      <c r="G24" s="10"/>
+      <c r="D23" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="E23" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="F23" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="G23" s="11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="49.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="B24" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="D24" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="E24" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="F24" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="G24" s="11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="69.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="B25" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="C25" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="D25" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="E25" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="F25" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="G25" s="11" t="s">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>